<commit_message>
fix: release the annex airlock safely during an emergency
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V159.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V159.xlsx
@@ -117,8 +117,8 @@
   <autoFilter ref="A5:E9"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Module"/>
-    <tableColumn id="2" name="SHA V157"/>
-    <tableColumn id="3" name="SHA V158"/>
+    <tableColumn id="2" name="SHA V158"/>
+    <tableColumn id="3" name="SHA V159"/>
     <tableColumn id="4" name="Évolution volontaire"/>
     <tableColumn id="5" name="Vérificateurs comportementaux"/>
   </tableColumns>
@@ -1694,12 +1694,12 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHA V157</t>
+          <t xml:space="preserve">SHA V158</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHA V158</t>
+          <t xml:space="preserve">SHA V159</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
@@ -1807,12 +1807,12 @@
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e015ad1958f6dec98149dd288023b0076ef0240ce72b788b38c7047c6acac407</t>
+          <t xml:space="preserve">320356c188b644ab4c47bf1a1ff786a15ad9b3501bdc08dac498645ffa409ed8</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contrôleur borné du même BISHOP, marche sur sols natifs et passage de sas apparié entièrement occulté avant changement de repère.</t>
+          <t xml:space="preserve">Contrôleur du même BISHOP sur sols natifs ; sas occulté, puis réouverture et retrait réel dans la pièce courante sous crise ou infestation avant libération du passage.</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
@@ -12994,7 +12994,7 @@
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Implémenté (trajet borné)</t>
+          <t xml:space="preserve">Implémenté (trajet borné ; sas dégagé physiquement sous alerte)</t>
         </is>
       </c>
       <c r="E6" s="0" t="inlineStr">
@@ -24494,7 +24494,7 @@
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Affectation native conditionnelle ; V159 suit le même BISHOP depuis science-lab par le sas apparié et le retour. Priorités mission/alerte/soins conservées ; pas de trajet quarantaine ou autres annexes.</t>
+          <t xml:space="preserve">Affectation native conditionnelle ; V159 suit le même BISHOP depuis science-lab par le sas apparié et le retour. Sous crise ou infestation au sas : réouverture, retrait dans la même pièce puis fermeture avant libération du passage. Missions et soins prioritaires ; pas de trajet quarantaine ou autres annexes.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: prioritize emergency door clearance over interaction timers
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V159.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V159.xlsx
@@ -1807,12 +1807,12 @@
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">320356c188b644ab4c47bf1a1ff786a15ad9b3501bdc08dac498645ffa409ed8</t>
+          <t xml:space="preserve">d079a3b5895e0bd7b32f5de3281b3dc3a9badc072544859ff16cb18c3e0a2306</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contrôleur du même BISHOP sur sols natifs ; sas occulté, puis réouverture et retrait réel dans la pièce courante sous crise ou infestation avant libération du passage.</t>
+          <t xml:space="preserve">Contrôleur du même BISHOP sur sols natifs ; sous crise ou infestation, réouverture et retrait réel dans la pièce courante avant libération du sas, y compris avec minuteurs d’interaction actifs.</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
@@ -24494,7 +24494,7 @@
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Affectation native conditionnelle ; V159 suit le même BISHOP depuis science-lab par le sas apparié et le retour. Sous crise ou infestation au sas : réouverture, retrait dans la même pièce puis fermeture avant libération du passage. Missions et soins prioritaires ; pas de trajet quarantaine ou autres annexes.</t>
+          <t xml:space="preserve">Affectation native conditionnelle ; V159 suit le même BISHOP depuis science-lab par le sas apparié et le retour. Sous crise ou infestation au sas, y compris avec minuteurs d’interaction actifs : réouverture, retrait dans la même pièce puis fermeture avant libération du passage. Missions et soins prioritaires ; pas de trajet quarantaine ou autres annexes.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: reserve the occupied aperture and animate emergency withdrawal
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V159.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V159.xlsx
@@ -1807,12 +1807,12 @@
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d079a3b5895e0bd7b32f5de3281b3dc3a9badc072544859ff16cb18c3e0a2306</t>
+          <t xml:space="preserve">5034808833beea323a3a3836c60cfeb40d5822575e085f0bead50d8826038f81</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contrôleur du même BISHOP sur sols natifs ; sous crise ou infestation, réouverture et retrait réel dans la pièce courante avant libération du sas, y compris avec minuteurs d’interaction actifs.</t>
+          <t xml:space="preserve">Même BISHOP sur sols natifs ; retrait d’alerte prioritaire aux minuteurs, ouverture recouverte réservée dès l’approche même à progression zéro, marche native pilotée par distance réelle.</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
@@ -12994,7 +12994,7 @@
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Implémenté (trajet borné ; sas dégagé physiquement sous alerte)</t>
+          <t xml:space="preserve">Implémenté (trajet borné ; réservation physique et marche native pendant le retrait d’alerte)</t>
         </is>
       </c>
       <c r="E6" s="0" t="inlineStr">
@@ -24494,7 +24494,7 @@
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Affectation native conditionnelle ; V159 suit le même BISHOP depuis science-lab par le sas apparié et le retour. Sous crise ou infestation au sas, y compris avec minuteurs d’interaction actifs : réouverture, retrait dans la même pièce puis fermeture avant libération du passage. Missions et soins prioritaires ; pas de trajet quarantaine ou autres annexes.</t>
+          <t xml:space="preserve">Affectation native conditionnelle ; V159 suit le même BISHOP depuis science-lab par le sas apparié et le retour. Alerte : retrait réel prioritaire aux minuteurs, réservation dès le corps sur l’ouverture même à progression zéro, marche native pilotée par distance. Missions et soins prioritaires ; quarantaine et autres annexes hors de ce circuit.</t>
         </is>
       </c>
     </row>

</xml_diff>